<commit_message>
updated to reflect 1944 lgs
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -1,3 +1,140 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
@@ -280,4 +417,464 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Model Level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Predictors</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>N (observations)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>DF (residuals)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DF (model)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>R-squared</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>F-value</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>P-value (F)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SSR</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SSTO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>MSE (model)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>MSE (residuals)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>MSE (total)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Beta coefs</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>P-values (beta coefs)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Std Beta coefs</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Partial correlations</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Semi-partial correlations</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Unique variance %</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>R-squared change</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>F-value change</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>P-value (F-value change)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>['N1ratio-ArgsPreds']</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>418</v>
+      </c>
+      <c r="E2" t="n">
+        <v>416</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2811745503463828</v>
+      </c>
+      <c r="H2" t="n">
+        <v>162.721858276525</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.103326246471194e-31</v>
+      </c>
+      <c r="J2" t="n">
+        <v>50.76489778415019</v>
+      </c>
+      <c r="K2" t="n">
+        <v>70.62200956937799</v>
+      </c>
+      <c r="L2" t="n">
+        <v>19.8571117852278</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.1220310042888226</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1693573370968297</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>{'const': 0.7246497473222122, 'N1ratio-ArgsPreds': -0.201038911394247}</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>{'const': 3.2085579622124637e-48, 'N1ratio-ArgsPreds': 1.1033262464710236e-31}</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': -0.5302589465029163}</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.530258946502916)}</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5302589465029159)}</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(28.117455034638226)}</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>['N1ratio-ArgsPreds', 'latitude', 'longitude', 'Macro_class']</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>418</v>
+      </c>
+      <c r="E3" t="n">
+        <v>413</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.3559952808179712</v>
+      </c>
+      <c r="H3" t="n">
+        <v>57.07491210800622</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.557531470181153e-38</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45.48090744079783</v>
+      </c>
+      <c r="K3" t="n">
+        <v>70.62200956937799</v>
+      </c>
+      <c r="L3" t="n">
+        <v>6.285275532145041</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.1101232625685177</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1693573370968297</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>{'const': 0.5965768578350408, 'N1ratio-ArgsPreds': -0.20787895370022813, 'latitude': 0.0053758004860521985, 'longitude': 7.114974965205078e-05, 'Macro_class': 0.04311930034831653}</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>{'const': 2.1808713790275152e-30, 'N1ratio-ArgsPreds': 8.780702031362679e-33, 'latitude': 4.7067850563177887e-08, 'longitude': 0.7522731057022538, 'Macro_class': 7.541683104730277e-06}</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': -0.5483001983285005, 'latitude': 0.22918570253720066, 'longitude': 0.013670090255655732, 'Macro_class': 0.18530480160725032}</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5399839572775078), 'latitude': np.float64(0.2641413846395274), 'longitude': np.float64(0.015540268024094611), 'Macro_class': np.float64(0.2178187242854485)}</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5148500924551618), 'latitude': np.float64(0.2197788825654119), 'longitude': np.float64(0.012472556419013996), 'Macro_class': np.float64(0.17909963625090008)}</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(26.507061770108862), 'latitude': np.float64(4.830275722170111), 'longitude': np.float64(0.015556466362548723), 'Macro_class': np.float64(3.2076679705204727)}</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>0.07482073047158833</v>
+      </c>
+      <c r="V3" t="n">
+        <v>15.99416938228563</v>
+      </c>
+      <c r="W3" t="n">
+        <v>7.430064375148832e-10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>['N1ratio-ArgsPreds', 'latitude', 'longitude', 'Macro_class', 'Fam_class']</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>418</v>
+      </c>
+      <c r="E4" t="n">
+        <v>412</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.3611063850808393</v>
+      </c>
+      <c r="H4" t="n">
+        <v>46.57295899635197</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.086902788203054e-38</v>
+      </c>
+      <c r="J4" t="n">
+        <v>45.11995098663547</v>
+      </c>
+      <c r="K4" t="n">
+        <v>70.62200956937799</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5.100411716548505</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.1095144441423191</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1693573370968297</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>{'const': 0.6166067283032032, 'N1ratio-ArgsPreds': -0.20042166090621383, 'latitude': 0.005385196489048594, 'longitude': -3.0008256834859222e-05, 'Macro_class': 0.04556846011453821, 'Fam_class': -0.0007593584976009544}</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>{'const': 7.241482284239388e-31, 'N1ratio-ArgsPreds': 1.861245449861111e-29, 'latitude': 4.1211410651777654e-08, 'longitude': 0.8969019842012975, 'Macro_class': 2.7034997684459866e-06, 'Fam_class': 0.07017687466421106}</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': -0.5286308905646754, 'latitude': 0.2295862809354053, 'longitude': -0.005765523861342213, 'Macro_class': 0.19583004345760624, 'Fam_class': -0.07530053741414049}</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5152973701424373), 'latitude': np.float64(0.2655490313288939), 'longitude': np.float64(-0.006387555243544143), 'Macro_class': np.float64(0.22824565869756938), 'Fam_class': np.float64(-0.08908669454503249)}</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4806020037313429), 'latitude': np.float64(0.2201598413500411), 'longitude': np.float64(-0.005105729509521445), 'Macro_class': np.float64(0.18738492114963518), 'Fam_class': np.float64(-0.0714919874032448)}</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(23.09782859905817), 'latitude': np.float64(4.847035574327527), 'longitude': np.float64(0.0026068473824398097), 'Macro_class': np.float64(3.511310867425499), 'Fam_class': np.float64(0.5111104262865713)}</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>0.005111104262868094</v>
+      </c>
+      <c r="V4" t="n">
+        <v>3.295971202604832</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.07017687466421452</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>['N1ratio-ArgsPreds', 'latitude', 'longitude', 'Macro_class', 'Fam_class', 'Nlen_freq', 'Vlen_freq']</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>418</v>
+      </c>
+      <c r="E5" t="n">
+        <v>410</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.3697426589285074</v>
+      </c>
+      <c r="H5" t="n">
+        <v>34.36113207411984</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.250128592015841e-37</v>
+      </c>
+      <c r="J5" t="n">
+        <v>44.51003997232168</v>
+      </c>
+      <c r="K5" t="n">
+        <v>70.62200956937799</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3.730281371008045</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.1085610731032236</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1693573370968297</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>{'const': 0.7013501340966837, 'N1ratio-ArgsPreds': -0.19403734177464727, 'latitude': 0.005577296079290736, 'longitude': -0.00011459859166858949, 'Macro_class': 0.04071234379715194, 'Fam_class': -0.0008737214168739748, 'Nlen_freq': -0.05940888885305038, 'Vlen_freq': 0.04811196355741011}</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>{'const': 2.9313250976475575e-12, 'N1ratio-ArgsPreds': 1.6203612207951728e-27, 'latitude': 1.368723282750051e-08, 'longitude': 0.624112382975412, 'Macro_class': 6.715766707073865e-05, 'Fam_class': 0.03932830469012555, 'Nlen_freq': 0.023989883485208658, 'Vlen_freq': 0.023069578590412455}</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': -0.5117916512683379, 'latitude': 0.2377760341937308, 'longitude': -0.022017970533161266, 'Macro_class': 0.17496092769028312, 'Fam_class': -0.0866411483491798, 'Nlen_freq': -0.16914534108338167, 'Vlen_freq': 0.17736994818507948}</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5005945471317725), 'latitude': np.float64(0.27511867636277954), 'longitude': np.float64(-0.024212087595894497), 'Macro_class': np.float64(0.19508554020467853), 'Fam_class': np.float64(-0.10157103836357542), 'Nlen_freq': np.float64(-0.11120149778073618), 'Vlen_freq': np.float64(0.11193528336704316)}</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4590782834627526), 'latitude': np.float64(0.22718009206846088), 'longitude': np.float64(-0.019227309955033862), 'Macro_class': np.float64(0.15791001562286588), 'Fam_class': np.float64(-0.0810551702707607), 'Nlen_freq': np.float64(-0.0888324269024948), 'Vlen_freq': np.float64(0.08942601868396126)}</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>{'N1ratio-ArgsPreds': np.float64(21.07528703471074), 'latitude': np.float64(5.161079423223436), 'longitude': np.float64(0.036968944810694425), 'Macro_class': np.float64(2.4935573034013747), 'Fam_class': np.float64(0.656994062762201), 'Nlen_freq': np.float64(0.7891200069387081), 'Vlen_freq': np.float64(0.7997012817664187)}</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0.008636273847668186</v>
+      </c>
+      <c r="V5" t="n">
+        <v>2.809068650849956</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.06142141887007796</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated scripts to include test data from Old Irish, updated wordlength readme
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2811745503463828</v>
+        <v>0.2718410704128487</v>
       </c>
       <c r="H2" t="n">
-        <v>162.721858276525</v>
+        <v>155.3038501579072</v>
       </c>
       <c r="I2" t="n">
-        <v>1.103326246471194e-31</v>
+        <v>1.641648662219235e-30</v>
       </c>
       <c r="J2" t="n">
-        <v>50.76489778415019</v>
+        <v>46.19802586758672</v>
       </c>
       <c r="K2" t="n">
-        <v>70.62200956937799</v>
+        <v>63.44497607655501</v>
       </c>
       <c r="L2" t="n">
-        <v>19.8571117852278</v>
+        <v>17.24695020896829</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1220310042888226</v>
+        <v>0.1110529467970835</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1693573370968297</v>
+        <v>0.1521462256032494</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.7246497473222122, 'N1ratio-ArgsPreds': -0.201038911394247}</t>
+          <t>{'const': 0.6853830788583233, 'N1ratio-ArgsPreds': -0.1969132311588327}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 3.2085579622124637e-48, 'N1ratio-ArgsPreds': 1.1033262464710236e-31}</t>
+          <t>{'const': 1.2134845764834344e-44, 'N1ratio-ArgsPreds': 1.6416486622189097e-30}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5302589465029163}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5213838033664343}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.530258946502916)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5213838033664335)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5302589465029159)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5213838033664336)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(28.117455034638226)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(27.184107041284793)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3559952808179712</v>
+        <v>0.336436176012663</v>
       </c>
       <c r="H3" t="n">
-        <v>57.07491210800622</v>
+        <v>52.34919975681247</v>
       </c>
       <c r="I3" t="n">
-        <v>2.557531470181153e-38</v>
+        <v>1.166291635171683e-35</v>
       </c>
       <c r="J3" t="n">
-        <v>45.48090744079783</v>
+        <v>42.09979093814395</v>
       </c>
       <c r="K3" t="n">
-        <v>70.62200956937799</v>
+        <v>63.44497607655501</v>
       </c>
       <c r="L3" t="n">
-        <v>6.285275532145041</v>
+        <v>5.336296284602764</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1101232625685177</v>
+        <v>0.1019365398018013</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1693573370968297</v>
+        <v>0.1521462256032494</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.5965768578350408, 'N1ratio-ArgsPreds': -0.20787895370022813, 'latitude': 0.0053758004860521985, 'longitude': 7.114974965205078e-05, 'Macro_class': 0.04311930034831653}</t>
+          <t>{'const': 0.5499752288880718, 'N1ratio-ArgsPreds': -0.19337507675445287, 'latitude': 0.0030823123906620316, 'longitude': -0.0003167259141907613, 'Macro_class': 0.05220467360411124}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 2.1808713790275152e-30, 'N1ratio-ArgsPreds': 8.780702031362679e-33, 'latitude': 4.7067850563177887e-08, 'longitude': 0.7522731057022538, 'Macro_class': 7.541683104730277e-06}</t>
+          <t>{'const': 1.0038730692171636e-27, 'N1ratio-ArgsPreds': 3.0995117976584226e-29, 'latitude': 0.001940551257214772, 'longitude': 0.1463903903879598, 'Macro_class': 2.2658115564941052e-08}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5483001983285005, 'latitude': 0.22918570253720066, 'longitude': 0.013670090255655732, 'Macro_class': 0.18530480160725032}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5120155329389116, 'latitude': 0.1304051059463067, 'longitude': -0.06394385744004548, 'Macro_class': 0.23572869715871117}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5399839572775078), 'latitude': np.float64(0.2641413846395274), 'longitude': np.float64(0.015540268024094611), 'Macro_class': np.float64(0.2178187242854485)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5130069858301057), 'latitude': np.float64(0.15170901292685426), 'longitude': np.float64(-0.07141986539513599), 'Macro_class': np.float64(0.2701177885614781)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5148500924551618), 'latitude': np.float64(0.2197788825654119), 'longitude': np.float64(0.012472556419013996), 'Macro_class': np.float64(0.17909963625090008)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.48683612550844296), 'latitude': np.float64(0.12502847216657229), 'longitude': np.float64(-0.05832716077228636), 'Macro_class': np.float64(0.2285315405429897)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(26.507061770108862), 'latitude': np.float64(4.830275722170111), 'longitude': np.float64(0.015556466362548723), 'Macro_class': np.float64(3.2076679705204727)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(23.70094131000724), 'latitude': np.float64(1.563211885230734), 'longitude': np.float64(0.3402057683756141), 'Macro_class': np.float64(5.222666502295214)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.07482073047158833</v>
+        <v>0.0645951055998143</v>
       </c>
       <c r="V3" t="n">
-        <v>15.99416938228563</v>
+        <v>13.40126231938387</v>
       </c>
       <c r="W3" t="n">
-        <v>7.430064375148832e-10</v>
+        <v>2.312803729721872e-08</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3611063850808393</v>
+        <v>0.336577317319246</v>
       </c>
       <c r="H4" t="n">
-        <v>46.57295899635197</v>
+        <v>41.80437550769086</v>
       </c>
       <c r="I4" t="n">
-        <v>4.086902788203054e-38</v>
+        <v>8.644209746465449e-35</v>
       </c>
       <c r="J4" t="n">
-        <v>45.11995098663547</v>
+        <v>42.09083623132438</v>
       </c>
       <c r="K4" t="n">
-        <v>70.62200956937799</v>
+        <v>63.44497607655501</v>
       </c>
       <c r="L4" t="n">
-        <v>5.100411716548505</v>
+        <v>4.270827969046126</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1095144441423191</v>
+        <v>0.1021622238624378</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1693573370968297</v>
+        <v>0.1521462256032494</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.6166067283032032, 'N1ratio-ArgsPreds': -0.20042166090621383, 'latitude': 0.005385196489048594, 'longitude': -3.0008256834859222e-05, 'Macro_class': 0.04556846011453821, 'Fam_class': -0.0007593584976009544}</t>
+          <t>{'const': 0.5527515166747254, 'N1ratio-ArgsPreds': -0.19200688877032324, 'latitude': 0.0030892888515746024, 'longitude': -0.0003338764112991427, 'Macro_class': 0.052588198328808955, 'Fam_class': -0.0001210307929581289}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 7.241482284239388e-31, 'N1ratio-ArgsPreds': 1.861245449861111e-29, 'latitude': 4.1211410651777654e-08, 'longitude': 0.8969019842012975, 'Macro_class': 2.7034997684459866e-06, 'Fam_class': 0.07017687466421106}</t>
+          <t>{'const': 5.1721469984201364e-27, 'N1ratio-ArgsPreds': 5.325456375050425e-27, 'latitude': 0.0019234421733749377, 'longitude': 0.1394233509035092, 'Macro_class': 2.5419376005933454e-08, 'Fam_class': 0.7673330226288387}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5286308905646754, 'latitude': 0.2295862809354053, 'longitude': -0.005765523861342213, 'Macro_class': 0.19583004345760624, 'Fam_class': -0.07530053741414049}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5083928659871395, 'latitude': 0.13070026296127707, 'longitude': -0.06740637469230838, 'Macro_class': 0.2374604919854875, 'Fam_class': -0.01266247246068786}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5152973701424373), 'latitude': np.float64(0.2655490313288939), 'longitude': np.float64(-0.006387555243544143), 'Macro_class': np.float64(0.22824565869756938), 'Fam_class': np.float64(-0.08908669454503249)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4952047185672786), 'latitude': np.float64(0.15201813470962988), 'longitude': np.float64(-0.07276056627145171), 'Macro_class': np.float64(0.2695020808897746), 'Fam_class': np.float64(-0.014584304262373499)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4806020037313429), 'latitude': np.float64(0.2201598413500411), 'longitude': np.float64(-0.005105729509521445), 'Macro_class': np.float64(0.18738492114963518), 'Fam_class': np.float64(-0.0714919874032448)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4642714303106744), 'latitude': np.float64(0.12527592475000354), 'longitude': np.float64(-0.05942153705321467), 'Macro_class': np.float64(0.22794553034330783), 'Fam_class': np.float64(-0.011880290677542281)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(23.09782859905817), 'latitude': np.float64(4.847035574327527), 'longitude': np.float64(0.0026068473824398097), 'Macro_class': np.float64(3.511310867425499), 'Fam_class': np.float64(0.5111104262865713)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(21.554796100271943), 'latitude': np.float64(1.569405732196855), 'longitude': np.float64(0.3530919065766564), 'Macro_class': np.float64(5.1959164803491875), 'Fam_class': np.float64(0.014114130658289802)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.005111104262868094</v>
+        <v>0.000141141306583048</v>
       </c>
       <c r="V4" t="n">
-        <v>3.295971202604832</v>
+        <v>0.08765183921243508</v>
       </c>
       <c r="W4" t="n">
-        <v>0.07017687466421452</v>
+        <v>0.7673330226287745</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3697426589285074</v>
+        <v>0.3426506647071466</v>
       </c>
       <c r="H5" t="n">
-        <v>34.36113207411984</v>
+        <v>30.53100970111432</v>
       </c>
       <c r="I5" t="n">
-        <v>1.250128592015841e-37</v>
+        <v>5.787899522596862e-34</v>
       </c>
       <c r="J5" t="n">
-        <v>44.51003997232168</v>
+        <v>41.70551285159442</v>
       </c>
       <c r="K5" t="n">
-        <v>70.62200956937799</v>
+        <v>63.44497607655501</v>
       </c>
       <c r="L5" t="n">
-        <v>3.730281371008045</v>
+        <v>3.105637603565798</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1085610731032236</v>
+        <v>0.1017207630526693</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1693573370968297</v>
+        <v>0.1521462256032494</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.7013501340966837, 'N1ratio-ArgsPreds': -0.19403734177464727, 'latitude': 0.005577296079290736, 'longitude': -0.00011459859166858949, 'Macro_class': 0.04071234379715194, 'Fam_class': -0.0008737214168739748, 'Nlen_freq': -0.05940888885305038, 'Vlen_freq': 0.04811196355741011}</t>
+          <t>{'const': 0.5484745904557893, 'N1ratio-ArgsPreds': -0.18684725744539568, 'latitude': 0.00315590946944603, 'longitude': -0.0003847273187767611, 'Macro_class': 0.04694337194305739, 'Fam_class': -0.00028415678787632514, 'Nlen_freq': -0.03411696735046287, 'Vlen_freq': 0.0374858081581514}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 2.9313250976475575e-12, 'N1ratio-ArgsPreds': 1.6203612207951728e-27, 'latitude': 1.368723282750051e-08, 'longitude': 0.624112382975412, 'Macro_class': 6.715766707073865e-05, 'Fam_class': 0.03932830469012555, 'Nlen_freq': 0.023989883485208658, 'Vlen_freq': 0.023069578590412455}</t>
+          <t>{'const': 1.3273686346593486e-09, 'N1ratio-ArgsPreds': 4.631592360014207e-25, 'latitude': 0.0015103729250882866, 'longitude': 0.09323726175451312, 'Macro_class': 2.7662780626879177e-06, 'Fam_class': 0.49581026998166844, 'Nlen_freq': 0.14160645800433677, 'Vlen_freq': 0.05372005108464598}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5117916512683379, 'latitude': 0.2377760341937308, 'longitude': -0.022017970533161266, 'Macro_class': 0.17496092769028312, 'Fam_class': -0.0866411483491798, 'Nlen_freq': -0.16914534108338167, 'Vlen_freq': 0.17736994818507948}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4947312740853265, 'latitude': 0.13351881852302075, 'longitude': -0.07767267445737074, 'Macro_class': 0.211971441336667, 'Fam_class': -0.029729025259268328, 'Nlen_freq': -0.10838709557042298, 'Vlen_freq': 0.14867208287441444}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5005945471317725), 'latitude': np.float64(0.27511867636277954), 'longitude': np.float64(-0.024212087595894497), 'Macro_class': np.float64(0.19508554020467853), 'Fam_class': np.float64(-0.10157103836357542), 'Nlen_freq': np.float64(-0.11120149778073618), 'Vlen_freq': np.float64(0.11193528336704316)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4793668421006606), 'latitude': np.float64(0.15582447180198095), 'longitude': np.float64(-0.08280636868273741), 'Macro_class': np.float64(0.228564592760893), 'Fam_class': np.float64(-0.03364795604450879), 'Nlen_freq': np.float64(-0.07253853631919949), 'Vlen_freq': np.float64(0.09511271820864826)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4590782834627526), 'latitude': np.float64(0.22718009206846088), 'longitude': np.float64(-0.019227309955033862), 'Macro_class': np.float64(0.15791001562286588), 'Fam_class': np.float64(-0.0810551702707607), 'Nlen_freq': np.float64(-0.0888324269024948), 'Vlen_freq': np.float64(0.08942601868396126)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4428557138505202), 'latitude': np.float64(0.12790026835215695), 'longitude': np.float64(-0.06736835423906654), 'Macro_class': np.float64(0.19035236925821458), 'Fam_class': np.float64(-0.02729623774843979), 'Nlen_freq': np.float64(-0.058967472440342686), 'Vlen_freq': np.float64(0.07746580781214177)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(21.07528703471074), 'latitude': np.float64(5.161079423223436), 'longitude': np.float64(0.036968944810694425), 'Macro_class': np.float64(2.4935573034013747), 'Fam_class': np.float64(0.656994062762201), 'Nlen_freq': np.float64(0.7891200069387081), 'Vlen_freq': np.float64(0.7997012817664187)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(19.612118329005384), 'latitude': np.float64(1.635847864455376), 'longitude': np.float64(0.4538495152880354), 'Macro_class': np.float64(3.6234024482215674), 'Fam_class': np.float64(0.07450845952193492), 'Nlen_freq': np.float64(0.34771628060025744), 'Vlen_freq': np.float64(0.6000951379987685)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.008636273847668186</v>
+        <v>0.006073347387900552</v>
       </c>
       <c r="V5" t="n">
-        <v>2.809068650849956</v>
+        <v>1.894025212583415</v>
       </c>
       <c r="W5" t="n">
-        <v>0.06142141887007796</v>
+        <v>0.1517790938257255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated readme, scripts, and output to reflect addition of re-tagged data
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2718410704128487</v>
+        <v>0.2245712216695587</v>
       </c>
       <c r="H2" t="n">
-        <v>155.3038501579072</v>
+        <v>120.4773808055982</v>
       </c>
       <c r="I2" t="n">
-        <v>1.641648662219235e-30</v>
+        <v>8.662773579461411e-25</v>
       </c>
       <c r="J2" t="n">
-        <v>46.19802586758672</v>
+        <v>47.72226153720241</v>
       </c>
       <c r="K2" t="n">
-        <v>63.44497607655501</v>
+        <v>61.54306220095695</v>
       </c>
       <c r="L2" t="n">
-        <v>17.24695020896829</v>
+        <v>13.82080066375454</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1110529467970835</v>
+        <v>0.1147169748490443</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1521462256032494</v>
+        <v>0.1475852810574507</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.6853830788583233, 'N1ratio-ArgsPreds': -0.1969132311588327}</t>
+          <t>{'const': 0.62499541565161, 'N1ratio-ArgsPreds': -0.18104180896765626}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 1.2134845764834344e-44, 'N1ratio-ArgsPreds': 1.6416486622189097e-30}</t>
+          <t>{'const': 7.985526650447148e-38, 'N1ratio-ArgsPreds': 8.662773579460338e-25}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5213838033664343}</t>
+          <t>{'N1ratio-ArgsPreds': -0.47388946144597743}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5213838033664335)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4738894614459782)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5213838033664336)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.47388946144597816)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(27.184107041284793)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.457122166955923)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.336436176012663</v>
+        <v>0.3092399628114294</v>
       </c>
       <c r="H3" t="n">
-        <v>52.34919975681247</v>
+        <v>46.2230361360117</v>
       </c>
       <c r="I3" t="n">
-        <v>1.166291635171683e-35</v>
+        <v>4.295676547311822e-32</v>
       </c>
       <c r="J3" t="n">
-        <v>42.09979093814395</v>
+        <v>42.51148793463154</v>
       </c>
       <c r="K3" t="n">
-        <v>63.44497607655501</v>
+        <v>61.54306220095695</v>
       </c>
       <c r="L3" t="n">
-        <v>5.336296284602764</v>
+        <v>4.757893566581354</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1019365398018013</v>
+        <v>0.1029333848296163</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1521462256032494</v>
+        <v>0.1475852810574507</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.5499752288880718, 'N1ratio-ArgsPreds': -0.19337507675445287, 'latitude': 0.0030823123906620316, 'longitude': -0.0003167259141907613, 'Macro_class': 0.05220467360411124}</t>
+          <t>{'const': 0.48471916730083336, 'N1ratio-ArgsPreds': -0.18947424649405237, 'latitude': 0.0021909270518130773, 'longitude': 0.00030277392346812125, 'Macro_class': 0.05826226118133984}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 1.0038730692171636e-27, 'N1ratio-ArgsPreds': 3.0995117976584226e-29, 'latitude': 0.001940551257214772, 'longitude': 0.1463903903879598, 'Macro_class': 2.2658115564941052e-08}</t>
+          <t>{'const': 2.2243285330241402e-22, 'N1ratio-ArgsPreds': 1.239675716612444e-26, 'latitude': 0.018856351180476953, 'longitude': 0.16002936481495172, 'Macro_class': 3.2865136033398286e-10}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5120155329389116, 'latitude': 0.1304051059463067, 'longitude': -0.06394385744004548, 'Macro_class': 0.23572869715871117}</t>
+          <t>{'N1ratio-ArgsPreds': -0.49596195012053884, 'latitude': 0.0995710723041759, 'longitude': 0.06263764817884489, 'Macro_class': 0.2700839444988631}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5130069858301057), 'latitude': np.float64(0.15170901292685426), 'longitude': np.float64(-0.07141986539513599), 'Macro_class': np.float64(0.2701177885614781)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4915677105213559), 'latitude': np.float64(0.11523969174313325), 'longitude': np.float64(0.06909336188314953), 'Macro_class': np.float64(0.3021705863199895)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.48683612550844296), 'latitude': np.float64(0.12502847216657229), 'longitude': np.float64(-0.05832716077228636), 'Macro_class': np.float64(0.2285315405429897)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.46914695440786114), 'latitude': np.float64(0.09642036374605199), 'longitude': np.float64(0.05756242036817744), 'Macro_class': np.float64(0.2634554658551867)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(23.70094131000724), 'latitude': np.float64(1.563211885230734), 'longitude': np.float64(0.3402057683756141), 'Macro_class': np.float64(5.222666502295214)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.009886483017173), 'latitude': np.float64(0.9296886544920977), 'longitude': np.float64(0.33134322386427695), 'Macro_class': np.float64(6.940878248897345)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.0645951055998143</v>
+        <v>0.08466874114187073</v>
       </c>
       <c r="V3" t="n">
-        <v>13.40126231938387</v>
+        <v>16.87425840571929</v>
       </c>
       <c r="W3" t="n">
-        <v>2.312803729721872e-08</v>
+        <v>2.337518692616245e-10</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.336577317319246</v>
+        <v>0.3111388636023295</v>
       </c>
       <c r="H4" t="n">
-        <v>41.80437550769086</v>
+        <v>37.21772213033015</v>
       </c>
       <c r="I4" t="n">
-        <v>8.644209746465449e-35</v>
+        <v>1.789005446304117e-31</v>
       </c>
       <c r="J4" t="n">
-        <v>42.09083623132438</v>
+        <v>42.39462376514373</v>
       </c>
       <c r="K4" t="n">
-        <v>63.44497607655501</v>
+        <v>61.54306220095695</v>
       </c>
       <c r="L4" t="n">
-        <v>4.270827969046126</v>
+        <v>3.829687687162645</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1021622238624378</v>
+        <v>0.1028995722454945</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1521462256032494</v>
+        <v>0.1475852810574507</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.5527515166747254, 'N1ratio-ArgsPreds': -0.19200688877032324, 'latitude': 0.0030892888515746024, 'longitude': -0.0003338764112991427, 'Macro_class': 0.052588198328808955, 'Fam_class': -0.0001210307929581289}</t>
+          <t>{'const': 0.4939149183448046, 'N1ratio-ArgsPreds': -0.18375953536320083, 'latitude': 0.0021819949829872684, 'longitude': 0.0002426261256271716, 'Macro_class': 0.05940232416294447, 'Fam_class': -0.0004385475130416342}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 5.1721469984201364e-27, 'N1ratio-ArgsPreds': 5.325456375050425e-27, 'latitude': 0.0019234421733749377, 'longitude': 0.1394233509035092, 'Macro_class': 2.5419376005933454e-08, 'Fam_class': 0.7673330226288387}</t>
+          <t>{'const': 1.8425929996820956e-22, 'N1ratio-ArgsPreds': 2.5749579687114053e-23, 'latitude': 0.019329579341445555, 'longitude': 0.2758493634344424, 'Macro_class': 2.015765907475661e-10, 'Fam_class': 0.28718457701093153}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5083928659871395, 'latitude': 0.13070026296127707, 'longitude': -0.06740637469230838, 'Macro_class': 0.2374604919854875, 'Fam_class': -0.01266247246068786}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4810032983286625, 'latitude': 0.09916513652911461, 'longitude': 0.050194315685944894, 'Macro_class': 0.2753688871153287, 'Fam_class': -0.04658524199268568}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4952047185672786), 'latitude': np.float64(0.15201813470962988), 'longitude': np.float64(-0.07276056627145171), 'Macro_class': np.float64(0.2695020808897746), 'Fam_class': np.float64(-0.014584304262373499)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4623331552853377), 'latitude': np.float64(0.1149274639449626), 'longitude': np.float64(0.05367906245539817), 'Macro_class': np.float64(0.30598040125505344), 'Fam_class': np.float64(-0.05243092691515269)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4642714303106744), 'latitude': np.float64(0.12527592475000354), 'longitude': np.float64(-0.05942153705321467), 'Macro_class': np.float64(0.22794553034330783), 'Fam_class': np.float64(-0.011880290677542281)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4327539985428786), 'latitude': np.float64(0.09602336611570338), 'longitude': np.float64(0.044616691667032166), 'Macro_class': np.float64(0.26675050758052854), 'Fam_class': np.float64(-0.04357637881810631)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(21.554796100271943), 'latitude': np.float64(1.569405732196855), 'longitude': np.float64(0.3530919065766564), 'Macro_class': np.float64(5.1959164803491875), 'Fam_class': np.float64(0.014114130658289802)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(18.727602325484977), 'latitude': np.float64(0.9220486840190412), 'longitude': np.float64(0.19906491753110175), 'Macro_class': np.float64(7.115583329446961), 'Fam_class': np.float64(0.18989007908991043)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.000141141306583048</v>
+        <v>0.001898900790900049</v>
       </c>
       <c r="V4" t="n">
-        <v>0.08765183921243508</v>
+        <v>1.135710935794731</v>
       </c>
       <c r="W4" t="n">
-        <v>0.7673330226287745</v>
+        <v>0.2871845770109519</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3426506647071466</v>
+        <v>0.3199350559460145</v>
       </c>
       <c r="H5" t="n">
-        <v>30.53100970111432</v>
+        <v>27.55479964182719</v>
       </c>
       <c r="I5" t="n">
-        <v>5.787899522596862e-34</v>
+        <v>5.173048014968049e-31</v>
       </c>
       <c r="J5" t="n">
-        <v>41.70551285159442</v>
+        <v>41.85327915260474</v>
       </c>
       <c r="K5" t="n">
-        <v>63.44497607655501</v>
+        <v>61.54306220095695</v>
       </c>
       <c r="L5" t="n">
-        <v>3.105637603565798</v>
+        <v>2.812826149764601</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1017207630526693</v>
+        <v>0.1020811686648896</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1521462256032494</v>
+        <v>0.1475852810574507</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.5484745904557893, 'N1ratio-ArgsPreds': -0.18684725744539568, 'latitude': 0.00315590946944603, 'longitude': -0.0003847273187767611, 'Macro_class': 0.04694337194305739, 'Fam_class': -0.00028415678787632514, 'Nlen_freq': -0.03411696735046287, 'Vlen_freq': 0.0374858081581514}</t>
+          <t>{'const': 0.49017860829746385, 'N1ratio-ArgsPreds': -0.1766332177943038, 'latitude': 0.002498495047567121, 'longitude': 0.00018671768825122054, 'Macro_class': 0.05172449145147411, 'Fam_class': -0.0007045235001433715, 'Nlen_freq': -0.04208244071390485, 'Vlen_freq': 0.04619566955168282}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 1.3273686346593486e-09, 'N1ratio-ArgsPreds': 4.631592360014207e-25, 'latitude': 0.0015103729250882866, 'longitude': 0.09323726175451312, 'Macro_class': 2.7662780626879177e-06, 'Fam_class': 0.49581026998166844, 'Nlen_freq': 0.14160645800433677, 'Vlen_freq': 0.05372005108464598}</t>
+          <t>{'const': 1.9579228075530144e-07, 'N1ratio-ArgsPreds': 2.34988294967048e-21, 'latitude': 0.007881033444544189, 'longitude': 0.4084762773021128, 'Macro_class': 1.814486653505597e-07, 'Fam_class': 0.09892304765728696, 'Nlen_freq': 0.08035788268507556, 'Vlen_freq': 0.02285495505510877}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4947312740853265, 'latitude': 0.13351881852302075, 'longitude': -0.07767267445737074, 'Macro_class': 0.211971441336667, 'Fam_class': -0.029729025259268328, 'Nlen_freq': -0.10838709557042298, 'Vlen_freq': 0.14867208287441444}</t>
+          <t>{'N1ratio-ArgsPreds': -0.46234966901466823, 'latitude': 0.11354911649251759, 'longitude': 0.038628018990144654, 'Macro_class': 0.23977707687881722, 'Fam_class': -0.07483886413146078, 'Nlen_freq': -0.13422496210147442, 'Vlen_freq': 0.18587103216037582}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4793668421006606), 'latitude': np.float64(0.15582447180198095), 'longitude': np.float64(-0.08280636868273741), 'Macro_class': np.float64(0.228564592760893), 'Fam_class': np.float64(-0.03364795604450879), 'Nlen_freq': np.float64(-0.07253853631919949), 'Vlen_freq': np.float64(0.09511271820864826)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.44424398879575927), 'latitude': np.float64(0.13074200799067826), 'longitude': np.float64(0.04082964261201017), 'Macro_class': np.float64(0.2535995641163286), 'Fam_class': np.float64(-0.0814068140310272), 'Nlen_freq': np.float64(-0.08624944548188845), 'Vlen_freq': np.float64(0.11211004380925156)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4428557138505202), 'latitude': np.float64(0.12790026835215695), 'longitude': np.float64(-0.06736835423906654), 'Macro_class': np.float64(0.19035236925821458), 'Fam_class': np.float64(-0.02729623774843979), 'Nlen_freq': np.float64(-0.058967472440342686), 'Vlen_freq': np.float64(0.07746580781214177)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.40891626509310275), 'latitude': np.float64(0.1087512444673696), 'longitude': np.float64(0.0336986941691425), 'Macro_class': np.float64(0.21620131869828624), 'Fam_class': np.float64(-0.06735654339373863), 'Nlen_freq': np.float64(-0.07139255012814912), 'Vlen_freq': np.float64(0.09303926339243432)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(19.612118329005384), 'latitude': np.float64(1.635847864455376), 'longitude': np.float64(0.4538495152880354), 'Macro_class': np.float64(3.6234024482215674), 'Fam_class': np.float64(0.07450845952193492), 'Nlen_freq': np.float64(0.34771628060025744), 'Vlen_freq': np.float64(0.6000951379987685)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(16.72125118576927), 'latitude': np.float64(1.1826833173201587), 'longitude': np.float64(0.11356019887053988), 'Macro_class': np.float64(4.6743010206877935), 'Fam_class': np.float64(0.4536903937952595), 'Nlen_freq': np.float64(0.5096896213800284), 'Vlen_freq': np.float64(0.8656304532606768)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.006073347387900552</v>
+        <v>0.008796192343685005</v>
       </c>
       <c r="V5" t="n">
-        <v>1.894025212583415</v>
+        <v>2.651540042199677</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1517790938257255</v>
+        <v>0.07175207354894722</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated script and results to use compling 2025 data
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2245712216695587</v>
+        <v>0.255605115792593</v>
       </c>
       <c r="H2" t="n">
-        <v>120.4773808055982</v>
+        <v>142.8431742689033</v>
       </c>
       <c r="I2" t="n">
-        <v>8.662773579461411e-25</v>
+        <v>1.661405041146207e-28</v>
       </c>
       <c r="J2" t="n">
-        <v>47.72226153720241</v>
+        <v>44.36451041955723</v>
       </c>
       <c r="K2" t="n">
-        <v>61.54306220095695</v>
+        <v>59.59808612440192</v>
       </c>
       <c r="L2" t="n">
-        <v>13.82080066375454</v>
+        <v>15.23357570484468</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1147169748490443</v>
+        <v>0.1066454577393203</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1475852810574507</v>
+        <v>0.1429210698426905</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.62499541565161, 'N1ratio-ArgsPreds': -0.18104180896765626}</t>
+          <t>{'const': 0.634537333307279, 'N1ratio-ArgsPreds': -0.18321299787625028}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 7.985526650447148e-38, 'N1ratio-ArgsPreds': 8.662773579460338e-25}</t>
+          <t>{'const': 1.1739859365544702e-41, 'N1ratio-ArgsPreds': 1.6614050411459064e-28}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.47388946144597743}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5055740458059462}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4738894614459782)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5055740458059467)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.47388946144597816)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5055740458059468)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.457122166955923)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(25.56051157925936)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3092399628114294</v>
+        <v>0.325462415078886</v>
       </c>
       <c r="H3" t="n">
-        <v>46.2230361360117</v>
+        <v>49.81782351064234</v>
       </c>
       <c r="I3" t="n">
-        <v>4.295676547311822e-32</v>
+        <v>3.338919235792955e-34</v>
       </c>
       <c r="J3" t="n">
-        <v>42.51148793463154</v>
+        <v>40.20114908027463</v>
       </c>
       <c r="K3" t="n">
-        <v>61.54306220095695</v>
+        <v>59.59808612440192</v>
       </c>
       <c r="L3" t="n">
-        <v>4.757893566581354</v>
+        <v>4.849234261031823</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1029333848296163</v>
+        <v>0.09733934402003541</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1475852810574507</v>
+        <v>0.1429210698426905</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.48471916730083336, 'N1ratio-ArgsPreds': -0.18947424649405237, 'latitude': 0.0021909270518130773, 'longitude': 0.00030277392346812125, 'Macro_class': 0.05826226118133984}</t>
+          <t>{'const': 0.5150327021555743, 'N1ratio-ArgsPreds': -0.1944448312543232, 'latitude': 0.003552190749306972, 'longitude': 0.00039055509567864323, 'Macro_class': 0.046356053099758744}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 2.2243285330241402e-22, 'N1ratio-ArgsPreds': 1.239675716612444e-26, 'latitude': 0.018856351180476953, 'longitude': 0.16002936481495172, 'Macro_class': 3.2865136033398286e-10}</t>
+          <t>{'const': 6.110170272482638e-26, 'N1ratio-ArgsPreds': 1.0908506848506459e-30, 'latitude': 0.0002279800985430862, 'longitude': 0.060615269249563536, 'Macro_class': 2.2974931474282775e-07}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.49596195012053884, 'latitude': 0.0995710723041759, 'longitude': 0.06263764817884489, 'Macro_class': 0.2700839444988631}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5365681538037101, 'latitude': 0.15668025893968465, 'longitude': 0.08243193229049767, 'Macro_class': 0.2187304838670592}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4915677105213559), 'latitude': np.float64(0.11523969174313325), 'longitude': np.float64(0.06909336188314953), 'Macro_class': np.float64(0.3021705863199895)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5243534984530581), 'latitude': np.float64(0.1799922023642654), 'longitude': np.float64(0.09218537366436236), 'Macro_class': np.float64(0.25064798247908987)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.46914695440786114), 'latitude': np.float64(0.09642036374605199), 'longitude': np.float64(0.05756242036817744), 'Macro_class': np.float64(0.2634554658551867)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5057574016669016), 'latitude': np.float64(0.1502824296723566), 'longitude': np.float64(0.07603583702284289), 'Macro_class': np.float64(0.21264579838962855)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.009886483017173), 'latitude': np.float64(0.9296886544920977), 'longitude': np.float64(0.33134322386427695), 'Macro_class': np.float64(6.940878248897345)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(25.579054934085566), 'latitude': np.float64(2.2584808668226812), 'longitude': np.float64(0.5781448511764326), 'Macro_class': np.float64(4.521823557276255)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.08466874114187073</v>
+        <v>0.06985729928629292</v>
       </c>
       <c r="V3" t="n">
-        <v>16.87425840571929</v>
+        <v>14.25720634411254</v>
       </c>
       <c r="W3" t="n">
-        <v>2.337518692616245e-10</v>
+        <v>7.39697334164411e-09</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3111388636023295</v>
+        <v>0.3281463320699682</v>
       </c>
       <c r="H4" t="n">
-        <v>37.21772213033015</v>
+        <v>40.24575447488859</v>
       </c>
       <c r="I4" t="n">
-        <v>1.789005446304117e-31</v>
+        <v>1.122586800538901e-33</v>
       </c>
       <c r="J4" t="n">
-        <v>42.39462376514373</v>
+        <v>40.04119276428936</v>
       </c>
       <c r="K4" t="n">
-        <v>61.54306220095695</v>
+        <v>59.59808612440192</v>
       </c>
       <c r="L4" t="n">
-        <v>3.829687687162645</v>
+        <v>3.911378672022512</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1028995722454945</v>
+        <v>0.09718736107837223</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1475852810574507</v>
+        <v>0.1429210698426905</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.4939149183448046, 'N1ratio-ArgsPreds': -0.18375953536320083, 'latitude': 0.0021819949829872684, 'longitude': 0.0002426261256271716, 'Macro_class': 0.05940232416294447, 'Fam_class': -0.0004385475130416342}</t>
+          <t>{'const': 0.5277711630734738, 'N1ratio-ArgsPreds': -0.18924533391455062, 'latitude': 0.0035875739503536384, 'longitude': 0.0003274855395885815, 'Macro_class': 0.04784483920998574, 'Fam_class': -0.0005059347316502225}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 1.8425929996820956e-22, 'N1ratio-ArgsPreds': 2.5749579687114053e-23, 'latitude': 0.019329579341445555, 'longitude': 0.2758493634344424, 'Macro_class': 2.015765907475661e-10, 'Fam_class': 0.28718457701093153}</t>
+          <t>{'const': 5.086185067052485e-26, 'N1ratio-ArgsPreds': 7.330725936417535e-28, 'latitude': 0.0001967405383202816, 'longitude': 0.1252363397488314, 'Macro_class': 1.1987819258495504e-07, 'Fam_class': 0.20024523918776008}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4810032983286625, 'latitude': 0.09916513652911461, 'longitude': 0.050194315685944894, 'Macro_class': 0.2753688871153287, 'Fam_class': -0.04658524199268568}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5222202039491827, 'latitude': 0.15824094345618708, 'longitude': 0.06912024993189515, 'Macro_class': 0.22575530337798091, 'Fam_class': -0.05461344738178258}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4623331552853377), 'latitude': np.float64(0.1149274639449626), 'longitude': np.float64(0.05367906245539817), 'Macro_class': np.float64(0.30598040125505344), 'Fam_class': np.float64(-0.05243092691515269)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5024013432472366), 'latitude': np.float64(0.1820033306954515), 'longitude': np.float64(0.07547141376274501), 'Macro_class': np.float64(0.25657798987008296), 'Fam_class': np.float64(-0.06307851537807825)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4327539985428786), 'latitude': np.float64(0.09602336611570338), 'longitude': np.float64(0.044616691667032166), 'Macro_class': np.float64(0.26675050758052854), 'Fam_class': np.float64(-0.04357637881810631)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4762725557308478), 'latitude': np.float64(0.15171606294085385), 'longitude': np.float64(0.06203834792606642), 'Macro_class': np.float64(0.21759269591329258), 'Fam_class': np.float64(-0.05180653425086476)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(18.727602325484977), 'latitude': np.float64(0.9220486840190412), 'longitude': np.float64(0.19906491753110175), 'Macro_class': np.float64(7.115583329446961), 'Fam_class': np.float64(0.18989007908991043)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.68355473423935), 'latitude': np.float64(2.3017763754273126), 'longitude': np.float64(0.38487566133956697), 'Macro_class': np.float64(4.734658131481462), 'Fam_class': np.float64(0.2683916991086024)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.001898900790900049</v>
+        <v>0.00268391699108228</v>
       </c>
       <c r="V4" t="n">
-        <v>1.135710935794731</v>
+        <v>1.645855121596295</v>
       </c>
       <c r="W4" t="n">
-        <v>0.2871845770109519</v>
+        <v>0.2002452391877431</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3199350559460145</v>
+        <v>0.3587354350530791</v>
       </c>
       <c r="H5" t="n">
-        <v>27.55479964182719</v>
+        <v>32.76595660948608</v>
       </c>
       <c r="I5" t="n">
-        <v>5.173048014968049e-31</v>
+        <v>4.036854530083345e-36</v>
       </c>
       <c r="J5" t="n">
-        <v>41.85327915260474</v>
+        <v>38.21814077023372</v>
       </c>
       <c r="K5" t="n">
-        <v>61.54306220095695</v>
+        <v>59.59808612440192</v>
       </c>
       <c r="L5" t="n">
-        <v>2.812826149764601</v>
+        <v>3.054277907738314</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1020811686648896</v>
+        <v>0.09321497748837491</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1475852810574507</v>
+        <v>0.1429210698426905</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.49017860829746385, 'N1ratio-ArgsPreds': -0.1766332177943038, 'latitude': 0.002498495047567121, 'longitude': 0.00018671768825122054, 'Macro_class': 0.05172449145147411, 'Fam_class': -0.0007045235001433715, 'Nlen_freq': -0.04208244071390485, 'Vlen_freq': 0.04619566955168282}</t>
+          <t>{'const': 0.6423783535314487, 'N1ratio-ArgsPreds': -0.17572217743991175, 'latitude': 0.0037766901799110367, 'longitude': 0.00014960606974252397, 'Macro_class': 0.04241820012500528, 'Fam_class': -0.0007470584621117057, 'Nlen_freq': -0.09080531130227106, 'Vlen_freq': 0.07473524092746966}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 1.9579228075530144e-07, 'N1ratio-ArgsPreds': 2.34988294967048e-21, 'latitude': 0.007881033444544189, 'longitude': 0.4084762773021128, 'Macro_class': 1.814486653505597e-07, 'Fam_class': 0.09892304765728696, 'Nlen_freq': 0.08035788268507556, 'Vlen_freq': 0.02285495505510877}</t>
+          <t>{'const': 3.064834765479048e-14, 'N1ratio-ArgsPreds': 9.8365738937601e-25, 'latitude': 6.536509713229383e-05, 'longitude': 0.48246932100340734, 'Macro_class': 5.7236247459018826e-06, 'Fam_class': 0.06086231261569046, 'Nlen_freq': 2.109375005474879e-05, 'Vlen_freq': 4.168463779447632e-05}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.46234966901466823, 'latitude': 0.11354911649251759, 'longitude': 0.038628018990144654, 'Macro_class': 0.23977707687881722, 'Fam_class': -0.07483886413146078, 'Nlen_freq': -0.13422496210147442, 'Vlen_freq': 0.18587103216037582}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4849032176534396, 'latitude': 0.16658249432096847, 'longitude': 0.031576383326491, 'Macro_class': 0.20014977155508618, 'Fam_class': -0.0806417022974017, 'Nlen_freq': -0.3213473112744426, 'Vlen_freq': 0.32278995329226434}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.44424398879575927), 'latitude': np.float64(0.13074200799067826), 'longitude': np.float64(0.04082964261201017), 'Macro_class': np.float64(0.2535995641163286), 'Fam_class': np.float64(-0.0814068140310272), 'Nlen_freq': np.float64(-0.08624944548188845), 'Vlen_freq': np.float64(0.11211004380925156)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.47642441909829925), 'latitude': np.float64(0.19539357219227926), 'longitude': np.float64(0.03469663356371136), 'Macro_class': np.float64(0.22138340658555772), 'Fam_class': np.float64(-0.09243275373689111), 'Nlen_freq': np.float64(-0.20786812772190072), 'Vlen_freq': np.float64(0.2004472754838539)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.40891626509310275), 'latitude': np.float64(0.1087512444673696), 'longitude': np.float64(0.0336986941691425), 'Macro_class': np.float64(0.21620131869828624), 'Fam_class': np.float64(-0.06735654339373863), 'Nlen_freq': np.float64(-0.07139255012814912), 'Vlen_freq': np.float64(0.09303926339243432)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4339276584784996), 'latitude': np.float64(0.1595444447574644), 'longitude': np.float64(0.02780145542925472), 'Macro_class': np.float64(0.18179245388793816), 'Fam_class': np.float64(-0.07433746540124178), 'Nlen_freq': np.float64(-0.1701758861383618), 'Vlen_freq': np.float64(0.1638414111606402)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(16.72125118576927), 'latitude': np.float64(1.1826833173201587), 'longitude': np.float64(0.11356019887053988), 'Macro_class': np.float64(4.6743010206877935), 'Fam_class': np.float64(0.4536903937952595), 'Nlen_freq': np.float64(0.5096896213800284), 'Vlen_freq': np.float64(0.8656304532606768)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(18.829321279263343), 'latitude': np.float64(2.545442985296761), 'longitude': np.float64(0.07729209239848368), 'Macro_class': np.float64(3.3048496290598126), 'Fam_class': np.float64(0.5526058762280819), 'Nlen_freq': np.float64(2.8959832222976676), 'Vlen_freq': np.float64(2.6844008011109954)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.008796192343685005</v>
+        <v>0.03058910298311091</v>
       </c>
       <c r="V5" t="n">
-        <v>2.651540042199677</v>
+        <v>9.778750385274732</v>
       </c>
       <c r="W5" t="n">
-        <v>0.07175207354894722</v>
+        <v>7.101052249424413e-05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated legend hue order for plots
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2132032938108851</v>
+        <v>0.2068012167026907</v>
       </c>
       <c r="H2" t="n">
-        <v>112.7261585205594</v>
+        <v>108.4586965586325</v>
       </c>
       <c r="I2" t="n">
-        <v>1.833955737282271e-23</v>
+        <v>1.004435449916872e-22</v>
       </c>
       <c r="J2" t="n">
-        <v>52.33703927174244</v>
+        <v>49.32254252503267</v>
       </c>
       <c r="K2" t="n">
-        <v>66.51913875598086</v>
+        <v>62.18181818181816</v>
       </c>
       <c r="L2" t="n">
-        <v>14.18209948423842</v>
+        <v>12.85927565678549</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1258101905570732</v>
+        <v>0.1185638041467131</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1595183183596663</v>
+        <v>0.1491170699803793</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.5962233407458759, 'N1ratio-ArgsPreds': -0.15741161637301737}</t>
+          <t>{'const': 0.5484975922590092, 'N1ratio-ArgsPreds': -0.14096877826605125}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 1.2829129858167587e-38, 'N1ratio-ArgsPreds': 1.833955737282047e-23}</t>
+          <t>{'const': 5.529973901041431e-37, 'N1ratio-ArgsPreds': 1.0044354499166375e-22}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4617394219804984}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4547540177971947}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.46173942198049805)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4547540177971949)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.46173942198049805)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.45475401779719493)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(21.320329381088445)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(20.68012167026915)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2978198351762127</v>
+        <v>0.2548364897908404</v>
       </c>
       <c r="H3" t="n">
-        <v>43.79203446975843</v>
+        <v>35.31019328028932</v>
       </c>
       <c r="I3" t="n">
-        <v>1.223223156293077e-30</v>
+        <v>2.235158370328403e-25</v>
       </c>
       <c r="J3" t="n">
-        <v>46.70841981561102</v>
+        <v>46.33562190755136</v>
       </c>
       <c r="K3" t="n">
-        <v>66.51913875598086</v>
+        <v>62.18181818181816</v>
       </c>
       <c r="L3" t="n">
-        <v>4.95267973509246</v>
+        <v>3.961549068566699</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1130954474954262</v>
+        <v>0.1121927891224004</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1595183183596663</v>
+        <v>0.1491170699803793</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.45636878322137653, 'N1ratio-ArgsPreds': -0.16452367744849117, 'latitude': 0.0041196267458860816, 'longitude': 5.050058729492285e-06, 'Macro_class': 0.05579654937521477}</t>
+          <t>{'const': 0.4504592378508506, 'N1ratio-ArgsPreds': -0.14577283583013662, 'latitude': 0.0036911972122575655, 'longitude': -3.722897572367933e-05, 'Macro_class': 0.03748896521676736}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 2.9203774203026966e-22, 'N1ratio-ArgsPreds': 1.4906005292238952e-25, 'latitude': 5.481156858905365e-05, 'longitude': 0.982222257046871, 'Macro_class': 7.216138136010343e-09}</t>
+          <t>{'const': 1.879136256466386e-22, 'N1ratio-ArgsPreds': 6.153648857544467e-23, 'latitude': 0.00027886044598178825, 'longitude': 0.8712670038861563, 'Macro_class': 9.462669112248416e-05}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.48260140819057196, 'latitude': 0.17512436275328672, 'longitude': 0.0009972602686150515, 'Macro_class': 0.24863813780882907}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4702515237404873, 'latitude': 0.16336579764684478, 'longitude': -0.007583059710252152, 'Macro_class': 0.17269399226172702}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4822039073939242), 'latitude': np.float64(0.1966819448018615), 'longitude': np.float64(0.0010971354125309401), 'Macro_class': np.float64(0.2791896015438114)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4582537812078881), 'latitude': np.float64(0.17751180284865792), 'longitude': np.float64(-0.007978627744090984), 'Macro_class': np.float64(0.1904559586066012)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.46123434901501803), 'latitude': np.float64(0.1680953265844287), 'longitude': np.float64(0.0009193582405802367), 'Macro_class': np.float64(0.24363828612171293)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.44505875334742717), 'latitude': np.float64(0.15570607347566057), 'longitude': np.float64(-0.0068875983997907595), 'Macro_class': np.float64(0.16747247848272032)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(21.273712471130747), 'latitude': np.float64(2.825603881952574), 'longitude': np.float64(8.452195745227885e-05), 'Macro_class': np.float64(5.935961446432565)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(19.807729393116603), 'latitude': np.float64(2.424438131720781), 'longitude': np.float64(0.004743901171680023), 'Macro_class': np.float64(2.804703104914522)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.08461654136532759</v>
+        <v>0.0480352730881497</v>
       </c>
       <c r="V3" t="n">
-        <v>16.58958452286965</v>
+        <v>8.874368964487337</v>
       </c>
       <c r="W3" t="n">
-        <v>3.395870322908322e-10</v>
+        <v>1.034575804855128e-05</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2992364252758501</v>
+        <v>0.2555332692226215</v>
       </c>
       <c r="H4" t="n">
-        <v>35.18602040985952</v>
+        <v>28.28325365454171</v>
       </c>
       <c r="I4" t="n">
-        <v>5.757157942925538e-30</v>
+        <v>1.179077274879562e-24</v>
       </c>
       <c r="J4" t="n">
-        <v>46.61418946221288</v>
+        <v>46.29229489561152</v>
       </c>
       <c r="K4" t="n">
-        <v>66.51913875598086</v>
+        <v>62.18181818181816</v>
       </c>
       <c r="L4" t="n">
-        <v>3.980989858753595</v>
+        <v>3.177904657241328</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1131412365587691</v>
+        <v>0.1123599390670182</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1595183183596663</v>
+        <v>0.1491170699803793</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.46673644300542255, 'N1ratio-ArgsPreds': -0.16039191847386244, 'latitude': 0.0041011722614907944, 'longitude': -4.8396575450587764e-05, 'Macro_class': 0.056909104987295955, 'Fam_class': -0.0003931878308166683}</t>
+          <t>{'const': 0.4586160035488994, 'N1ratio-ArgsPreds': -0.14373232203636846, 'latitude': 0.003708300495974394, 'longitude': -7.190609570371391e-05, 'Macro_class': 0.03830587728206569, 'Fam_class': -0.00026270059582948074}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 6.5929250387380325e-22, 'N1ratio-ArgsPreds': 1.0044945088033547e-22, 'latitude': 5.952272598506861e-05, 'longitude': 0.836243085096272, 'Macro_class': 4.9597247561163755e-09, 'Fam_class': 0.3619816956204327}</t>
+          <t>{'const': 1.727390459183886e-21, 'N1ratio-ArgsPreds': 2.1707439156867093e-21, 'latitude': 0.000265664141809031, 'longitude': 0.7612053829790042, 'Macro_class': 7.893957497022484e-05, 'Fam_class': 0.5349599205823985}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.470481616496248, 'latitude': 0.17433986696786333, 'longitude': -0.009557112980100736, 'Macro_class': 0.25359585936498513, 'Fam_class': -0.04017427178008066}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4636689892424201, 'latitude': 0.16412275844468605, 'longitude': -0.014646339488345171, 'Macro_class': 0.1764571210935691, 'Fam_class': -0.027761990653456085}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4567113238049418), 'latitude': np.float64(0.19598726952301768), 'longitude': np.float64(-0.01018936233342405), 'Macro_class': np.float64(0.28242070113002143), 'Fam_class': np.float64(-0.04491566380255724)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.443622540200516), 'latitude': np.float64(0.17832451104636), 'longitude': np.float64(-0.014980240985692115), 'Macro_class': np.float64(0.192773881669266), 'Fam_class': np.float64(-0.030578900881027105)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.429759479260651), 'latitude': np.float64(0.16730883725002776), 'longitude': np.float64(-0.008530123358600214), 'Macro_class': np.float64(0.2464518462158015), 'Fam_class': np.float64(-0.03763761548819981)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4270951706210175), 'latitude': np.float64(0.15636914706988325), 'longitude': np.float64(-0.012926774774331918), 'Macro_class': np.float64(0.1695095521860099), 'Fam_class': np.float64(-0.026396579925824986)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(18.46932100143859), 'latitude': np.float64(2.799224702195628), 'longitude': np.float64(0.0072763004512937), 'Macro_class': np.float64(6.0738512503177065), 'Fam_class': np.float64(0.14165900996375785)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(18.241028476779604), 'latitude': np.float64(2.445131015536278), 'longitude': np.float64(0.016710150606630402), 'Macro_class': np.float64(2.873348828230162), 'Fam_class': np.float64(0.06967794317804667)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.00141659009963746</v>
+        <v>0.0006967794317811471</v>
       </c>
       <c r="V4" t="n">
-        <v>0.8328559618418767</v>
+        <v>0.3856090729455007</v>
       </c>
       <c r="W4" t="n">
-        <v>0.3619816956204396</v>
+        <v>0.5349599205823907</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3202594437606807</v>
+        <v>0.2764395065067559</v>
       </c>
       <c r="H5" t="n">
-        <v>27.59590105721148</v>
+        <v>22.37747493856586</v>
       </c>
       <c r="I5" t="n">
-        <v>4.702760163436519e-31</v>
+        <v>1.194570136465721e-25</v>
       </c>
       <c r="J5" t="n">
-        <v>45.21575637855089</v>
+        <v>44.99230704994353</v>
       </c>
       <c r="K5" t="n">
-        <v>66.51913875598086</v>
+        <v>62.18181818181816</v>
       </c>
       <c r="L5" t="n">
-        <v>3.043340339632853</v>
+        <v>2.455644447410662</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1102823326306119</v>
+        <v>0.1097373342681549</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1595183183596663</v>
+        <v>0.1491170699803793</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.5370081813098921, 'N1ratio-ArgsPreds': -0.15088423521849403, 'latitude': 0.004256077437900921, 'longitude': -0.0001896737157211686, 'Macro_class': 0.05334607663092741, 'Fam_class': -0.0007229060905657981, 'Nlen_freq': -0.07304560622315392, 'Vlen_freq': 0.06524430801429132}</t>
+          <t>{'const': 0.6294063036095336, 'N1ratio-ArgsPreds': -0.13867892824292305, 'latitude': 0.003820876833797703, 'longitude': -0.0002513946958071985, 'Macro_class': 0.037947036755347, 'Fam_class': -0.0004485199345600372, 'Nlen_freq': -0.07517304737915685, 'Vlen_freq': 0.05082509484435815}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 1.7166972750373872e-09, 'N1ratio-ArgsPreds': 2.024202812781739e-20, 'latitude': 2.5767437069365786e-05, 'longitude': 0.42098034574177157, 'Macro_class': 1.7141395098873254e-07, 'Fam_class': 0.10385808494777114, 'Nlen_freq': 0.0008464035954499458, 'Vlen_freq': 0.00073275127907}</t>
+          <t>{'const': 4.911398491136044e-11, 'N1ratio-ArgsPreds': 2.85030823144692e-20, 'latitude': 0.0001512284176055896, 'longitude': 0.29517824688662914, 'Macro_class': 0.0001844487715404442, 'Fam_class': 0.2957044976725832, 'Nlen_freq': 0.0006375585914970419, 'Vlen_freq': 0.007420446994921906}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4425924919712552, 'latitude': 0.18092484953530075, 'longitude': -0.03745581404522089, 'Macro_class': 0.2377184485679466, 'Fam_class': -0.07386349087545259, 'Nlen_freq': -0.2462133851084179, 'Vlen_freq': 0.26018059481061806}</t>
+          <t>{'N1ratio-ArgsPreds': -0.44736714454072607, 'latitude': 0.16910518614147588, 'longitude': -0.05120584039958269, 'Macro_class': 0.17480411192711082, 'Fam_class': -0.047399231021261055, 'Nlen_freq': -0.24715936364535307, 'Vlen_freq': 0.20032462766185177}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.43469630907325096), 'latitude': np.float64(0.20571538946162013), 'longitude': np.float64(-0.039750888553894116), 'Macro_class': np.float64(0.2540945722211396), 'Fam_class': np.float64(-0.08024302597707726), 'Nlen_freq': np.float64(-0.16379581274503116), 'Vlen_freq': np.float64(0.16572556960510332)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4331506383761294), 'latitude': np.float64(0.18561211062671062), 'longitude': np.float64(-0.0516961582859534), 'Macro_class': np.float64(0.18322255163296575), 'Fam_class': np.float64(-0.051639929754001605), 'Nlen_freq': np.float64(-0.16756844123379608), 'Vlen_freq': np.float64(0.13172910969637427)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.3979574532854041), 'latitude': np.float64(0.17331170605755908), 'longitude': np.float64(-0.032799092311053525), 'Macro_class': np.float64(0.21660074774013852), 'Fam_class': np.float64(-0.0663714962889807), 'Nlen_freq': np.float64(-0.13689255283384308), 'Vlen_freq': np.float64(0.138550623268803)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.40878658029106985), 'latitude': np.float64(0.1606781288479219), 'longitude': np.float64(-0.04403284990079908), 'Macro_class': np.float64(0.15853722854049646), 'Fam_class': np.float64(-0.043984828416780385), 'Nlen_freq': np.float64(-0.14458199423800663), 'Vlen_freq': np.float64(0.11303692010463381)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(15.837013462540458), 'latitude': np.float64(3.003694745658176), 'longitude': np.float64(0.10757804564290104), 'Macro_class': np.float64(4.691588392158712), 'Fam_class': np.float64(0.440517551963818), 'Nlen_freq': np.float64(1.873957102136652), 'Vlen_freq': np.float64(1.9196275208173772)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(16.71064682260673), 'latitude': np.float64(2.5817461090069393), 'longitude': np.float64(0.19388918703863015), 'Macro_class': np.float64(2.5134052833301603), 'Fam_class': np.float64(0.1934665130853611), 'Nlen_freq': np.float64(2.090395305783898), 'Vlen_freq': np.float64(1.2777345306741368)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.02102301848483057</v>
+        <v>0.02090623728413432</v>
       </c>
       <c r="V5" t="n">
-        <v>6.34024077249986</v>
+        <v>5.92317944634653</v>
       </c>
       <c r="W5" t="n">
-        <v>0.00194173945045655</v>
+        <v>0.002911106684066416</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-run scripts to check results
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_XX_All_lg_families_random_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2068012167026907</v>
+        <v>0.1910402142102136</v>
       </c>
       <c r="H2" t="n">
-        <v>108.4586965586325</v>
+        <v>98.24064249851392</v>
       </c>
       <c r="I2" t="n">
-        <v>1.004435449916872e-22</v>
+        <v>6.252852018520304e-21</v>
       </c>
       <c r="J2" t="n">
-        <v>49.32254252503267</v>
+        <v>51.82955029482362</v>
       </c>
       <c r="K2" t="n">
-        <v>62.18181818181816</v>
+        <v>64.06937799043062</v>
       </c>
       <c r="L2" t="n">
-        <v>12.85927565678549</v>
+        <v>12.239827695607</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1185638041467131</v>
+        <v>0.1245902651317875</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1491170699803793</v>
+        <v>0.1536435923031909</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.5484975922590092, 'N1ratio-ArgsPreds': -0.14096877826605125}</t>
+          <t>{'const': 0.5444440190341313, 'N1ratio-ArgsPreds': -0.13656564019229578}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 5.529973901041431e-37, 'N1ratio-ArgsPreds': 1.0044354499166375e-22}</t>
+          <t>{'const': 1.9574408011768344e-35, 'N1ratio-ArgsPreds': 6.2528520185195394e-21}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4547540177971947}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4370814731948878}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4547540177971949)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.43708147319488755)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.45475401779719493)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.43708147319488744)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(20.68012167026915)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(19.10402142102131)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2548364897908404</v>
+        <v>0.2663965756891696</v>
       </c>
       <c r="H3" t="n">
-        <v>35.31019328028932</v>
+        <v>37.49361784365473</v>
       </c>
       <c r="I3" t="n">
-        <v>2.235158370328403e-25</v>
+        <v>9.247859923855883e-27</v>
       </c>
       <c r="J3" t="n">
-        <v>46.33562190755136</v>
+        <v>47.00151508724485</v>
       </c>
       <c r="K3" t="n">
-        <v>62.18181818181816</v>
+        <v>64.06937799043062</v>
       </c>
       <c r="L3" t="n">
-        <v>3.961549068566699</v>
+        <v>4.266965725796442</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1121927891224004</v>
+        <v>0.1138051212766219</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1491170699803793</v>
+        <v>0.1536435923031909</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.4504592378508506, 'N1ratio-ArgsPreds': -0.14577283583013662, 'latitude': 0.0036911972122575655, 'longitude': -3.722897572367933e-05, 'Macro_class': 0.03748896521676736}</t>
+          <t>{'const': 0.4227498709668022, 'N1ratio-ArgsPreds': -0.14961615850934934, 'latitude': 0.0038916229112357314, 'longitude': 0.0001356746269489299, 'Macro_class': 0.05364493172713713}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 1.879136256466386e-22, 'N1ratio-ArgsPreds': 6.153648857544467e-23, 'latitude': 0.00027886044598178825, 'longitude': 0.8712670038861563, 'Macro_class': 9.462669112248416e-05}</t>
+          <t>{'const': 1.126346602090595e-20, 'N1ratio-ArgsPreds': 7.22578302911965e-24, 'latitude': 0.00022010442299618603, 'longitude': 0.5459933936492543, 'Macro_class': 3.010293904384751e-08}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4702515237404873, 'latitude': 0.16336579764684478, 'longitude': -0.007583059710252152, 'Macro_class': 0.17269399226172702}</t>
+          <t>{'N1ratio-ArgsPreds': -0.478849957302184, 'latitude': 0.16737075180335467, 'longitude': 0.027779986868987652, 'Macro_class': 0.24351197143506093}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4582537812078881), 'latitude': np.float64(0.17751180284865792), 'longitude': np.float64(-0.007978627744090984), 'Macro_class': np.float64(0.1904559586066012)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4669890118977731), 'latitude': np.float64(0.18042173382892354), 'longitude': np.float64(0.029721235847669378), 'Macro_class': np.float64(0.2678126243404989)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.44505875334742717), 'latitude': np.float64(0.15570607347566057), 'longitude': np.float64(-0.0068875983997907595), 'Macro_class': np.float64(0.16747247848272032)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4523304507303168), 'latitude': np.float64(0.15711068127112324), 'longitude': np.float64(0.025467683329461425), 'Macro_class': np.float64(0.23808008335528108)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(19.807729393116603), 'latitude': np.float64(2.424438131720781), 'longitude': np.float64(0.004743901171680023), 'Macro_class': np.float64(2.804703104914522)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(20.460283665789156), 'latitude': np.float64(2.4683766169476473), 'longitude': np.float64(0.06486028941697274), 'Macro_class': np.float64(5.668212609045758)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.0480352730881497</v>
+        <v>0.07535636147895608</v>
       </c>
       <c r="V3" t="n">
-        <v>8.874368964487337</v>
+        <v>14.14123592277667</v>
       </c>
       <c r="W3" t="n">
-        <v>1.034575804855128e-05</v>
+        <v>8.629950234112579e-09</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2555332692226215</v>
+        <v>0.2695339516663859</v>
       </c>
       <c r="H4" t="n">
-        <v>28.28325365454171</v>
+        <v>30.40469528731165</v>
       </c>
       <c r="I4" t="n">
-        <v>1.179077274879562e-24</v>
+        <v>2.553480773322397e-26</v>
       </c>
       <c r="J4" t="n">
-        <v>46.29229489561152</v>
+        <v>46.80050535986248</v>
       </c>
       <c r="K4" t="n">
-        <v>62.18181818181816</v>
+        <v>64.06937799043062</v>
       </c>
       <c r="L4" t="n">
-        <v>3.177904657241328</v>
+        <v>3.453774526113628</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1123599390670182</v>
+        <v>0.1135934596113167</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1491170699803793</v>
+        <v>0.1536435923031909</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.4586160035488994, 'N1ratio-ArgsPreds': -0.14373232203636846, 'latitude': 0.003708300495974394, 'longitude': -7.190609570371391e-05, 'Macro_class': 0.03830587728206569, 'Fam_class': -0.00026270059582948074}</t>
+          <t>{'const': 0.4399441825909999, 'N1ratio-ArgsPreds': -0.14441489474137653, 'latitude': 0.003832587808324488, 'longitude': 6.0700182184802765e-05, 'Macro_class': 0.05499163640096681, 'Fam_class': -0.0005694861808105765}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 1.727390459183886e-21, 'N1ratio-ArgsPreds': 2.1707439156867093e-21, 'latitude': 0.000265664141809031, 'longitude': 0.7612053829790042, 'Macro_class': 7.893957497022484e-05, 'Fam_class': 0.5349599205823985}</t>
+          <t>{'const': 1.4012609767602125e-20, 'N1ratio-ArgsPreds': 3.660476059928484e-21, 'latitude': 0.0002730451437427287, 'longitude': 0.7931106160881429, 'Macro_class': 1.6169304996185902e-08, 'Fam_class': 0.18417318708823008}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4636689892424201, 'latitude': 0.16412275844468605, 'longitude': -0.014646339488345171, 'Macro_class': 0.1764571210935691, 'Fam_class': -0.027761990653456085}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4622031929551664, 'latitude': 0.1648317726210408, 'longitude': 0.012428633871782897, 'Macro_class': 0.24962510644160965, 'Fam_class': -0.05928969144647761}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.443622540200516), 'latitude': np.float64(0.17832451104636), 'longitude': np.float64(-0.014980240985692115), 'Macro_class': np.float64(0.192773881669266), 'Fam_class': np.float64(-0.030578900881027105)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.44133970249728227), 'latitude': np.float64(0.17798524227958926), 'longitude': np.float64(0.012928588872509113), 'Macro_class': np.float64(0.27314623418987805), 'Fam_class': np.float64(-0.06539621432592985)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4270951706210175), 'latitude': np.float64(0.15636914706988325), 'longitude': np.float64(-0.012926774774331918), 'Macro_class': np.float64(0.1695095521860099), 'Fam_class': np.float64(-0.026396579925824986)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4203547278487577), 'latitude': np.float64(0.15458746642273669), 'longitude': np.float64(0.011050640267111592), 'Macro_class': np.float64(0.24267920721760247), 'Fam_class': np.float64(-0.056012284163534654)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(18.241028476779604), 'latitude': np.float64(2.445131015536278), 'longitude': np.float64(0.016710150606630402), 'Macro_class': np.float64(2.873348828230162), 'Fam_class': np.float64(0.06967794317804667)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(17.669809722480316), 'latitude': np.float64(2.389728477500074), 'longitude': np.float64(0.012211665031310815), 'Macro_class': np.float64(5.889319761576404), 'Fam_class': np.float64(0.3137375977216555)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.0006967794317811471</v>
+        <v>0.003137375977216306</v>
       </c>
       <c r="V4" t="n">
-        <v>0.3856090729455007</v>
+        <v>1.769553705558085</v>
       </c>
       <c r="W4" t="n">
-        <v>0.5349599205823907</v>
+        <v>0.1841731870882475</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2764395065067559</v>
+        <v>0.2834751659915784</v>
       </c>
       <c r="H5" t="n">
-        <v>22.37747493856586</v>
+        <v>23.17232376129261</v>
       </c>
       <c r="I5" t="n">
-        <v>1.194570136465721e-25</v>
+        <v>1.714293738569893e-26</v>
       </c>
       <c r="J5" t="n">
-        <v>44.99230704994353</v>
+        <v>45.90730042961612</v>
       </c>
       <c r="K5" t="n">
-        <v>62.18181818181816</v>
+        <v>64.06937799043062</v>
       </c>
       <c r="L5" t="n">
-        <v>2.455644447410662</v>
+        <v>2.594582508687786</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1097373342681549</v>
+        <v>0.1119690254380881</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1491170699803793</v>
+        <v>0.1536435923031909</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.6294063036095336, 'N1ratio-ArgsPreds': -0.13867892824292305, 'latitude': 0.003820876833797703, 'longitude': -0.0002513946958071985, 'Macro_class': 0.037947036755347, 'Fam_class': -0.0004485199345600372, 'Nlen_freq': -0.07517304737915685, 'Vlen_freq': 0.05082509484435815}</t>
+          <t>{'const': 0.5369157685486179, 'N1ratio-ArgsPreds': -0.13882421180100757, 'latitude': 0.004048474919154379, 'longitude': -2.613892594556332e-05, 'Macro_class': 0.050501182140323016, 'Fam_class': -0.0007918341396589168, 'Nlen_freq': -0.0654152397439957, 'Vlen_freq': 0.05335397550276621}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 4.911398491136044e-11, 'N1ratio-ArgsPreds': 2.85030823144692e-20, 'latitude': 0.0001512284176055896, 'longitude': 0.29517824688662914, 'Macro_class': 0.0001844487715404442, 'Fam_class': 0.2957044976725832, 'Nlen_freq': 0.0006375585914970419, 'Vlen_freq': 0.007420446994921906}</t>
+          <t>{'const': 4.433912393518878e-09, 'N1ratio-ArgsPreds': 1.3166816637444056e-19, 'latitude': 0.00011584811448170356, 'longitude': 0.9102412425723977, 'Macro_class': 5.616183230064287e-07, 'Fam_class': 0.07152296512546417, 'Nlen_freq': 0.006221854422903922, 'Vlen_freq': 0.008080810516440388}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.44736714454072607, 'latitude': 0.16910518614147588, 'longitude': -0.05120584039958269, 'Macro_class': 0.17480411192711082, 'Fam_class': -0.047399231021261055, 'Nlen_freq': -0.24715936364535307, 'Vlen_freq': 0.20032462766185177}</t>
+          <t>{'N1ratio-ArgsPreds': -0.444310083588116, 'latitude': 0.17411663625465001, 'longitude': -0.005352062031543451, 'Macro_class': 0.22924145910638177, 'Fam_class': -0.08243852686704618, 'Nlen_freq': -0.21849933554522608, 'Vlen_freq': 0.22105001868724772}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4331506383761294), 'latitude': np.float64(0.18561211062671062), 'longitude': np.float64(-0.0516961582859534), 'Macro_class': np.float64(0.18322255163296575), 'Fam_class': np.float64(-0.051639929754001605), 'Nlen_freq': np.float64(-0.16756844123379608), 'Vlen_freq': np.float64(0.13172910969637427)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.42614091705695917), 'latitude': np.float64(0.1887732682547259), 'longitude': np.float64(-0.005570900670141224), 'Macro_class': np.float64(0.24354602945518558), 'Fam_class': np.float64(-0.08887944920233647), 'Nlen_freq': np.float64(-0.13458106774127898), 'Vlen_freq': np.float64(0.13032979261175634)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.40878658029106985), 'latitude': np.float64(0.1606781288479219), 'longitude': np.float64(-0.04403284990079908), 'Macro_class': np.float64(0.15853722854049646), 'Fam_class': np.float64(-0.043984828416780385), 'Nlen_freq': np.float64(-0.14458199423800663), 'Vlen_freq': np.float64(0.11303692010463381)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.3987355976511522), 'latitude': np.float64(0.16271795464774894), 'longitude': np.float64(-0.0047157174730431675), 'Macro_class': np.float64(0.21255654942147667), 'Fam_class': np.float64(-0.07553342124351675), 'Nlen_freq': np.float64(-0.11496579082934162), 'Vlen_freq': np.float64(0.11127034745435671)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(16.71064682260673), 'latitude': np.float64(2.5817461090069393), 'longitude': np.float64(0.19388918703863015), 'Macro_class': np.float64(2.5134052833301603), 'Fam_class': np.float64(0.1934665130853611), 'Nlen_freq': np.float64(2.090395305783898), 'Vlen_freq': np.float64(1.2777345306741368)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(15.899007683422154), 'latitude': np.float64(2.647713276474688), 'longitude': np.float64(0.002223799128556464), 'Macro_class': np.float64(4.518028670196466), 'Fam_class': np.float64(0.5705297724750548), 'Nlen_freq': np.float64(1.321713306101593), 'Vlen_freq': np.float64(1.2381090222613267)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.02090623728413432</v>
+        <v>0.01394121432519246</v>
       </c>
       <c r="V5" t="n">
-        <v>5.92317944634653</v>
+        <v>3.988625098555711</v>
       </c>
       <c r="W5" t="n">
-        <v>0.002911106684066416</v>
+        <v>0.0192485715575749</v>
       </c>
     </row>
   </sheetData>

</xml_diff>